<commit_message>
Pricing: block owner vacation 30.10.-16.11. (whole-period offer only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171K8tMkvKpu6ZM9fEvYkFu
</commit_message>
<xml_diff>
--- a/airbnb-pricing/output/preisplan.xlsx
+++ b/airbnb-pricing/output/preisplan.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G62"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -964,450 +964,454 @@
       <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" t="n">
-        <v>99</v>
-      </c>
-      <c r="E20" t="n">
-        <v>119</v>
-      </c>
-      <c r="F20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-17</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-18</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>209</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>219</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>MEDICA + COMPAMED 2026</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>2026-10-31</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>2026-10-31</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" t="n">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>MEDICA + COMPAMED 2026 + Tokio Hotel (Konzert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-21</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E21" t="n">
+      <c r="E22" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F21" t="n">
-        <v>2</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>2026-11-01</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="n">
-        <v>69</v>
-      </c>
-      <c r="E22" t="n">
-        <v>89</v>
-      </c>
-      <c r="F22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-22</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" t="n">
+        <v>69</v>
+      </c>
+      <c r="E23" t="n">
+        <v>89</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-11-26</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" t="n">
         <v>79</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E24" t="n">
         <v>99</v>
       </c>
-      <c r="F23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-05</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland Cup (Eishockey)</t>
-        </is>
-      </c>
+      <c r="F24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-27</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-28</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D25" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-11-29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-11-29</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>69</v>
+      </c>
+      <c r="E26" t="n">
+        <v>89</v>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E27" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="E25" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland Cup (Eishockey)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-08</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-08</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Deutschland Cup (Eishockey)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>2026-11-09</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-11-10</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" t="n">
-        <v>79</v>
-      </c>
-      <c r="E27" t="n">
-        <v>99</v>
-      </c>
-      <c r="F27" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>VALVE WORLD EXPO 2026</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="E28" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-05</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="F28" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Karnevalsauftakt 11.11.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-11-12</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" t="n">
-        <v>79</v>
-      </c>
-      <c r="E29" t="n">
-        <v>99</v>
-      </c>
-      <c r="F29" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="E29" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-11-13</t>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="C30" t="n">
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="E30" t="n">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-12-07</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-11-14</t>
+          <t>2026-12-09</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D31" t="n">
+        <v>69</v>
+      </c>
+      <c r="E31" t="n">
+        <v>89</v>
+      </c>
+      <c r="F31" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-12-10</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>79</v>
+      </c>
+      <c r="E32" t="n">
         <v>99</v>
       </c>
-      <c r="E31" t="n">
-        <v>119</v>
-      </c>
-      <c r="F31" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-15</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-15</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>189</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>199</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>MEDICA + COMPAMED 2026</t>
-        </is>
-      </c>
+      <c r="F32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2026-11-18</t>
+          <t>2026-12-11</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>209</v>
+        <v>99</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>219</v>
+        <v>119</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>MEDICA + COMPAMED 2026</t>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-12</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-12</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="2" t="n">
+        <v>109</v>
+      </c>
+      <c r="E34" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="E34" s="2" t="n">
-        <v>139</v>
-      </c>
       <c r="F34" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>MEDICA + COMPAMED 2026 + Tokio Hotel (Konzert)</t>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-21</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="E35" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-12-13</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" t="n">
+        <v>59</v>
+      </c>
+      <c r="E35" t="n">
+        <v>79</v>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-12-14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-11-22</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D36" t="n">
         <v>69</v>
@@ -1423,16 +1427,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D37" t="n">
         <v>79</v>
@@ -1448,683 +1452,334 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-11-27</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-11-28</t>
+          <t>2026-12-18</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-19</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-19</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E38" s="2" t="n">
+      <c r="E39" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>2026-11-29</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>2026-11-29</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>59</v>
+      </c>
+      <c r="E40" t="n">
+        <v>79</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-12-21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-12-21</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
         <v>69</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E41" t="n">
         <v>89</v>
       </c>
-      <c r="F39" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-03</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D40" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>VALVE WORLD EXPO 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>2026-12-22</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-12-05</t>
+          <t>2026-12-23</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-24</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-24</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="E44" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E42" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>2026-12-06</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>2026-12-06</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
-      </c>
-      <c r="D43" t="n">
-        <v>59</v>
-      </c>
-      <c r="E43" t="n">
-        <v>79</v>
-      </c>
-      <c r="F43" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2026-12-07</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>2026-12-09</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" t="n">
-        <v>69</v>
-      </c>
-      <c r="E44" t="n">
-        <v>89</v>
-      </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="F44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026 + Broilers – Santa's Action Club + Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>2026-12-10</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
-        <v>79</v>
-      </c>
-      <c r="E45" t="n">
-        <v>99</v>
-      </c>
-      <c r="F45" t="n">
-        <v>2</v>
-      </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="F45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026 + Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-27</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-12-11</t>
+          <t>2026-12-28</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-12-29</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-12-29</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>69</v>
+      </c>
+      <c r="E47" t="n">
+        <v>89</v>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E48" s="2" t="n">
         <v>119</v>
       </c>
-      <c r="F46" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-12</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-12</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-12-13</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>2026-12-13</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" t="n">
-        <v>59</v>
-      </c>
-      <c r="E48" t="n">
-        <v>79</v>
-      </c>
-      <c r="F48" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="F48" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Silvester</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-12-14</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>3</v>
-      </c>
-      <c r="D49" t="n">
-        <v>69</v>
-      </c>
-      <c r="E49" t="n">
-        <v>89</v>
-      </c>
-      <c r="F49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>2026-12-17</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>2026-12-17</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="n">
-        <v>79</v>
-      </c>
-      <c r="E50" t="n">
-        <v>99</v>
-      </c>
-      <c r="F50" t="n">
-        <v>2</v>
-      </c>
-      <c r="G50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-18</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-18</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D51" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E51" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-19</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-19</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="E52" s="2" t="n">
-        <v>129</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="n">
-        <v>59</v>
-      </c>
-      <c r="E53" t="n">
-        <v>79</v>
-      </c>
-      <c r="F53" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="n">
-        <v>69</v>
-      </c>
-      <c r="E54" t="n">
-        <v>89</v>
-      </c>
-      <c r="F54" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-22</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="E55" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="F55" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-24</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-24</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="E56" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-25</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-25</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="E57" s="2" t="n">
-        <v>109</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026 + Broilers – Santa's Action Club + Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-26</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-26</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="E58" s="2" t="n">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2" t="n">
         <v>139</v>
       </c>
-      <c r="F58" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026 + Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-27</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-28</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2026-12-29</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>2026-12-29</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" t="n">
-        <v>69</v>
-      </c>
-      <c r="E60" t="n">
-        <v>89</v>
-      </c>
-      <c r="F60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-30</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-30</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E61" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F61" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>Silvester</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="2" t="n">
-        <v>139</v>
-      </c>
-      <c r="E62" s="2" t="n">
+      <c r="E49" s="2" t="n">
         <v>159</v>
       </c>
-      <c r="F62" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
+      <c r="F49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>Silvester</t>
         </is>
@@ -5864,12 +5519,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Saison 1.08; Wochentag 1.12; Schulferien NRW (-3%); Nachfrageindex 1.17</t>
+          <t>Saison 1.08; Wochentag 1.12; Schulferien NRW (-3%); Nachfrageindex 1.17; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -5901,12 +5556,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Saison 1.08; Wochentag 1.15; Vorabend Allerheiligen (+3%); Schulferien NRW (-3%); Nachfrageindex 1.28</t>
+          <t>Saison 1.08; Wochentag 1.15; Vorabend Allerheiligen (+3%); Schulferien NRW (-3%); Nachfrageindex 1.28; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -5938,12 +5593,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.88; Allerheiligen (+0%); Nachfrageindex 0.88</t>
+          <t>Saison 1.00; Wochentag 0.88; Allerheiligen (+0%); Nachfrageindex 0.88; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -5975,12 +5630,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.95; Nachfrageindex 0.95</t>
+          <t>Saison 1.00; Wochentag 0.95; Nachfrageindex 0.95; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6012,12 +5667,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97</t>
+          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6049,12 +5704,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97</t>
+          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6090,12 +5745,12 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.05</t>
+          <t>Saison 1.00; Wochentag 1.00; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.05; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6131,12 +5786,12 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.12; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.18</t>
+          <t>Saison 1.00; Wochentag 1.12; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.18; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6172,12 +5827,12 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.15; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.21</t>
+          <t>Saison 1.00; Wochentag 1.15; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 1.21; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6213,12 +5868,12 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.88; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 0.92</t>
+          <t>Saison 1.00; Wochentag 0.88; Event: Deutschland Cup (Eishockey) (+5%); Nachfrageindex 0.92; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6250,12 +5905,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.95; Nachfrageindex 0.95</t>
+          <t>Saison 1.00; Wochentag 0.95; Nachfrageindex 0.95; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6287,12 +5942,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97</t>
+          <t>Saison 1.00; Wochentag 0.97; Nachfrageindex 0.97; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6328,12 +5983,12 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 0.97; Event: Karnevalsauftakt 11.11. (+12%); Nachfrageindex 1.09</t>
+          <t>Saison 1.00; Wochentag 0.97; Event: Karnevalsauftakt 11.11. (+12%); Nachfrageindex 1.09; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6365,12 +6020,12 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Nachfrageindex 1.00</t>
+          <t>Saison 1.00; Wochentag 1.00; Nachfrageindex 1.00; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6402,12 +6057,12 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.12; Nachfrageindex 1.12</t>
+          <t>Saison 1.00; Wochentag 1.12; Nachfrageindex 1.12; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6439,12 +6094,12 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.15; Nachfrageindex 1.15</t>
+          <t>Saison 1.00; Wochentag 1.15; Nachfrageindex 1.15; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6480,12 +6135,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+96%); Nachfrageindex 1.96</t>
+          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+96%); Nachfrageindex 1.96; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -6521,12 +6176,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>freigeben</t>
+          <t>blockiert</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+120%); Nachfrageindex 2.20</t>
+          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+120%); Nachfrageindex 2.20; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
         </is>
       </c>
     </row>
@@ -14147,13 +13802,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>9.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D4" t="n">
-        <v>1207</v>
+        <v>1113</v>
       </c>
       <c r="E4" t="n">
-        <v>1073</v>
+        <v>990</v>
       </c>
     </row>
     <row r="5">
@@ -14168,13 +13823,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>11</v>
+        <v>5.2</v>
       </c>
       <c r="D5" t="n">
-        <v>1435</v>
+        <v>716</v>
       </c>
       <c r="E5" t="n">
-        <v>1276</v>
+        <v>636</v>
       </c>
     </row>
     <row r="6">
@@ -14399,13 +14054,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>78.3</v>
+        <v>71.8</v>
       </c>
       <c r="D16" t="n">
-        <v>9193</v>
+        <v>8380</v>
       </c>
       <c r="E16" t="n">
-        <v>8172</v>
+        <v>7450</v>
       </c>
     </row>
     <row r="17">
@@ -14420,13 +14075,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13.6</v>
+        <v>12.5</v>
       </c>
       <c r="D17" t="n">
-        <v>1725</v>
+        <v>1590</v>
       </c>
       <c r="E17" t="n">
-        <v>1533</v>
+        <v>1414</v>
       </c>
     </row>
     <row r="18">
@@ -14441,13 +14096,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>15.6</v>
+        <v>7.5</v>
       </c>
       <c r="D18" t="n">
-        <v>2050</v>
+        <v>1023</v>
       </c>
       <c r="E18" t="n">
-        <v>1822</v>
+        <v>909</v>
       </c>
     </row>
     <row r="19">
@@ -14672,13 +14327,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>111.8</v>
+        <v>102.6</v>
       </c>
       <c r="D29" t="n">
-        <v>13132</v>
+        <v>11971</v>
       </c>
       <c r="E29" t="n">
-        <v>11675</v>
+        <v>10642</v>
       </c>
     </row>
     <row r="30">
@@ -14693,13 +14348,13 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>17.1</v>
+        <v>15.7</v>
       </c>
       <c r="D30" t="n">
-        <v>2156</v>
+        <v>1988</v>
       </c>
       <c r="E30" t="n">
-        <v>1917</v>
+        <v>1767</v>
       </c>
     </row>
     <row r="31">
@@ -14714,13 +14369,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>19.1</v>
+        <v>9.1</v>
       </c>
       <c r="D31" t="n">
-        <v>2466</v>
+        <v>1229</v>
       </c>
       <c r="E31" t="n">
-        <v>2193</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="32">
@@ -14945,13 +14600,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>139.4</v>
+        <v>128</v>
       </c>
       <c r="D42" t="n">
-        <v>16320</v>
+        <v>14915</v>
       </c>
       <c r="E42" t="n">
-        <v>14508</v>
+        <v>13259</v>
       </c>
     </row>
     <row r="43"/>

</xml_diff>

<commit_message>
Pricing: owner returns 15.11. - MEDICA nights available again
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171K8tMkvKpu6ZM9fEvYkFu
</commit_message>
<xml_diff>
--- a/airbnb-pricing/output/preisplan.xlsx
+++ b/airbnb-pricing/output/preisplan.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -966,22 +966,22 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2026-11-17</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2026-11-18</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>209</v>
+        <v>189</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>219</v>
+        <v>199</v>
       </c>
       <c r="F20" s="2" t="n">
         <v>3</v>
@@ -995,296 +995,300 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-18</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>129</v>
+        <v>209</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>139</v>
+        <v>219</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>3</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>MEDICA + COMPAMED 2026 + Tokio Hotel (Konzert)</t>
+          <t>MEDICA + COMPAMED 2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-19</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>129</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>MEDICA + COMPAMED 2026 + Tokio Hotel (Konzert)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>2026-11-20</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>2026-11-21</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="2" t="n">
+      <c r="C23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E23" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="F23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-11-22</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-11-22</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" t="n">
-        <v>69</v>
-      </c>
-      <c r="E23" t="n">
-        <v>89</v>
-      </c>
-      <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-11-22</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="n">
+        <v>69</v>
+      </c>
+      <c r="E24" t="n">
+        <v>89</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>2026-11-23</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>2026-11-26</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C25" t="n">
         <v>4</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>79</v>
       </c>
-      <c r="E24" t="n">
+      <c r="E25" t="n">
         <v>99</v>
       </c>
-      <c r="F24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="F25" t="n">
+        <v>2</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>2026-11-27</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>2026-11-28</t>
         </is>
       </c>
-      <c r="C25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="n">
+      <c r="C26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="E26" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="F26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>2026-11-29</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>2026-11-29</t>
         </is>
       </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="n">
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" t="n">
         <v>69</v>
       </c>
-      <c r="E26" t="n">
+      <c r="E27" t="n">
         <v>89</v>
       </c>
-      <c r="F26" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-03</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>VALVE WORLD EXPO 2026</t>
-        </is>
-      </c>
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-11-30</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>2026-12-04</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D28" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="E28" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="E28" s="2" t="n">
-        <v>119</v>
-      </c>
       <c r="F28" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+          <t>VALVE WORLD EXPO 2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-04</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>2026-12-05</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>2026-12-05</t>
         </is>
       </c>
-      <c r="C29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="2" t="n">
+      <c r="C30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="E30" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F29" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2026-12-06</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026-12-06</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>59</v>
-      </c>
-      <c r="E30" t="n">
-        <v>79</v>
-      </c>
-      <c r="F30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-12-07</t>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-12-09</t>
+          <t>2026-12-06</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D31" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E31" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F31" t="n">
         <v>1</v>
@@ -1294,130 +1298,130 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>2026-12-07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-12-09</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>69</v>
+      </c>
+      <c r="E32" t="n">
+        <v>89</v>
+      </c>
+      <c r="F32" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>2026-12-10</t>
         </is>
       </c>
-      <c r="C32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" t="n">
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
         <v>79</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E33" t="n">
         <v>99</v>
       </c>
-      <c r="F32" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-11</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-11</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
+      <c r="F33" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-11</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>2026-12-12</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>2026-12-12</t>
         </is>
       </c>
-      <c r="C34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="2" t="n">
+      <c r="C35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>2026-12-13</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>2026-12-13</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" t="n">
-        <v>59</v>
-      </c>
-      <c r="E35" t="n">
-        <v>79</v>
-      </c>
-      <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-12-14</t>
+          <t>2026-12-13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-12-13</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E36" t="n">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="F36" t="n">
         <v>1</v>
@@ -1427,184 +1431,180 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>2026-12-14</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>69</v>
+      </c>
+      <c r="E37" t="n">
+        <v>89</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>2026-12-17</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>2026-12-17</t>
         </is>
       </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" t="n">
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" t="n">
         <v>79</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E38" t="n">
         <v>99</v>
       </c>
-      <c r="F37" t="n">
-        <v>2</v>
-      </c>
-      <c r="G37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-18</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-18</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
-        </is>
-      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-18</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>2026-12-19</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>2026-12-19</t>
         </is>
       </c>
-      <c r="C39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="n">
+      <c r="C40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="E39" s="2" t="n">
+      <c r="E40" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="F39" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="F40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Düsseldorfer Weihnachtsmarkt 2026</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>2026-12-20</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="n">
-        <v>59</v>
-      </c>
-      <c r="E40" t="n">
-        <v>79</v>
-      </c>
-      <c r="F40" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-12-20</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>59</v>
+      </c>
+      <c r="E41" t="n">
+        <v>79</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>2026-12-21</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>2026-12-21</t>
         </is>
       </c>
-      <c r="C41" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" t="n">
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
         <v>69</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E42" t="n">
         <v>89</v>
       </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-22</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-23</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Weihnachten – Familienbesuche</t>
-        </is>
-      </c>
+      <c r="F42" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-12-24</t>
+          <t>2026-12-22</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-12-24</t>
+          <t>2026-12-23</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="F43" s="2" t="n">
         <v>2</v>
@@ -1618,168 +1618,197 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-24</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-12-25</t>
+          <t>2026-12-24</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D44" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="E44" s="2" t="n">
         <v>89</v>
       </c>
-      <c r="E44" s="2" t="n">
-        <v>109</v>
-      </c>
       <c r="F44" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026 + Broilers – Santa's Action Club + Weihnachten – Familienbesuche</t>
+          <t>Weihnachten – Familienbesuche</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-12-26</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-12-26</t>
+          <t>2026-12-25</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>119</v>
+        <v>89</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>139</v>
+        <v>109</v>
       </c>
       <c r="F45" s="2" t="n">
         <v>2</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Düsseldorfer Weihnachtsmarkt 2026 + Weihnachten – Familienbesuche</t>
+          <t>Düsseldorfer Weihnachtsmarkt 2026 + Broilers – Santa's Action Club + Weihnachten – Familienbesuche</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-26</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Düsseldorfer Weihnachtsmarkt 2026 + Weihnachten – Familienbesuche</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>2026-12-27</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>2026-12-28</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" s="2" t="n">
+      <c r="C47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="2" t="n">
         <v>69</v>
       </c>
-      <c r="E46" s="2" t="n">
+      <c r="E47" s="2" t="n">
         <v>89</v>
       </c>
-      <c r="F46" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="F47" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>Weihnachten – Familienbesuche</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>2026-12-29</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>2026-12-29</t>
         </is>
       </c>
-      <c r="C47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" t="n">
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
         <v>69</v>
       </c>
-      <c r="E47" t="n">
+      <c r="E48" t="n">
         <v>89</v>
       </c>
-      <c r="F47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-30</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>2026-12-30</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D48" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>119</v>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>Silvester</t>
-        </is>
-      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-30</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Silvester</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="C49" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="2" t="n">
+      <c r="C50" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="2" t="n">
         <v>139</v>
       </c>
-      <c r="E49" s="2" t="n">
+      <c r="E50" s="2" t="n">
         <v>159</v>
       </c>
-      <c r="F49" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
+      <c r="F50" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>Silvester</t>
         </is>
@@ -6135,12 +6164,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>blockiert</t>
+          <t>freigeben</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+96%); Nachfrageindex 1.96; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
+          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+96%); Nachfrageindex 1.96</t>
         </is>
       </c>
     </row>
@@ -6176,12 +6205,12 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>blockiert</t>
+          <t>freigeben</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+120%); Nachfrageindex 2.20; blockiert (Urlaub) – nur als Gesamtzeitraum vermietbar</t>
+          <t>Saison 1.00; Wochentag 1.00; Event: MEDICA + COMPAMED 2026 (+120%); Nachfrageindex 2.20</t>
         </is>
       </c>
     </row>
@@ -13823,13 +13852,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5.2</v>
+        <v>6.4</v>
       </c>
       <c r="D5" t="n">
-        <v>716</v>
+        <v>962</v>
       </c>
       <c r="E5" t="n">
-        <v>636</v>
+        <v>855</v>
       </c>
     </row>
     <row r="6">
@@ -14054,13 +14083,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>71.8</v>
+        <v>73</v>
       </c>
       <c r="D16" t="n">
-        <v>8380</v>
+        <v>8626</v>
       </c>
       <c r="E16" t="n">
-        <v>7450</v>
+        <v>7669</v>
       </c>
     </row>
     <row r="17">
@@ -14096,13 +14125,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>7.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="D18" t="n">
-        <v>1023</v>
+        <v>1375</v>
       </c>
       <c r="E18" t="n">
-        <v>909</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="19">
@@ -14327,13 +14356,13 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>102.6</v>
+        <v>104.2</v>
       </c>
       <c r="D29" t="n">
-        <v>11971</v>
+        <v>12323</v>
       </c>
       <c r="E29" t="n">
-        <v>10642</v>
+        <v>10955</v>
       </c>
     </row>
     <row r="30">
@@ -14369,13 +14398,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9.1</v>
+        <v>11</v>
       </c>
       <c r="D31" t="n">
-        <v>1229</v>
+        <v>1622</v>
       </c>
       <c r="E31" t="n">
-        <v>1093</v>
+        <v>1442</v>
       </c>
     </row>
     <row r="32">
@@ -14600,13 +14629,13 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>128</v>
+        <v>129.9</v>
       </c>
       <c r="D42" t="n">
-        <v>14915</v>
+        <v>15308</v>
       </c>
       <c r="E42" t="n">
-        <v>13259</v>
+        <v>13609</v>
       </c>
     </row>
     <row r="43"/>

</xml_diff>

<commit_message>
Pricing: payout ratio from actual booking (18.44% host fee incl. VAT)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0171K8tMkvKpu6ZM9fEvYkFu
</commit_message>
<xml_diff>
--- a/airbnb-pricing/output/preisplan.xlsx
+++ b/airbnb-pricing/output/preisplan.xlsx
@@ -15235,7 +15235,7 @@
         <v>954</v>
       </c>
       <c r="E4" t="n">
-        <v>848</v>
+        <v>778</v>
       </c>
     </row>
     <row r="5">
@@ -15256,7 +15256,7 @@
         <v>956</v>
       </c>
       <c r="E5" t="n">
-        <v>850</v>
+        <v>780</v>
       </c>
     </row>
     <row r="6">
@@ -15277,7 +15277,7 @@
         <v>884</v>
       </c>
       <c r="E6" t="n">
-        <v>786</v>
+        <v>721</v>
       </c>
     </row>
     <row r="7">
@@ -15298,7 +15298,7 @@
         <v>376</v>
       </c>
       <c r="E7" t="n">
-        <v>334</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8">
@@ -15319,7 +15319,7 @@
         <v>374</v>
       </c>
       <c r="E8" t="n">
-        <v>333</v>
+        <v>305</v>
       </c>
     </row>
     <row r="9">
@@ -15340,7 +15340,7 @@
         <v>280</v>
       </c>
       <c r="E9" t="n">
-        <v>249</v>
+        <v>228</v>
       </c>
     </row>
     <row r="10">
@@ -15361,7 +15361,7 @@
         <v>219</v>
       </c>
       <c r="E10" t="n">
-        <v>194</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11">
@@ -15382,7 +15382,7 @@
         <v>114</v>
       </c>
       <c r="E11" t="n">
-        <v>101</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12">
@@ -15403,7 +15403,7 @@
         <v>1251</v>
       </c>
       <c r="E12" t="n">
-        <v>1112</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="13">
@@ -15424,7 +15424,7 @@
         <v>943</v>
       </c>
       <c r="E13" t="n">
-        <v>839</v>
+        <v>769</v>
       </c>
     </row>
     <row r="14">
@@ -15445,7 +15445,7 @@
         <v>812</v>
       </c>
       <c r="E14" t="n">
-        <v>722</v>
+        <v>663</v>
       </c>
     </row>
     <row r="15">
@@ -15466,7 +15466,7 @@
         <v>1137</v>
       </c>
       <c r="E15" t="n">
-        <v>1010</v>
+        <v>927</v>
       </c>
     </row>
     <row r="16">
@@ -15487,7 +15487,7 @@
         <v>8301</v>
       </c>
       <c r="E16" t="n">
-        <v>7380</v>
+        <v>6771</v>
       </c>
     </row>
     <row r="17">
@@ -15508,7 +15508,7 @@
         <v>1363</v>
       </c>
       <c r="E17" t="n">
-        <v>1212</v>
+        <v>1112</v>
       </c>
     </row>
     <row r="18">
@@ -15529,7 +15529,7 @@
         <v>1366</v>
       </c>
       <c r="E18" t="n">
-        <v>1215</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="19">
@@ -15550,7 +15550,7 @@
         <v>1263</v>
       </c>
       <c r="E19" t="n">
-        <v>1123</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="20">
@@ -15571,7 +15571,7 @@
         <v>537</v>
       </c>
       <c r="E20" t="n">
-        <v>478</v>
+        <v>438</v>
       </c>
     </row>
     <row r="21">
@@ -15592,7 +15592,7 @@
         <v>535</v>
       </c>
       <c r="E21" t="n">
-        <v>475</v>
+        <v>436</v>
       </c>
     </row>
     <row r="22">
@@ -15613,7 +15613,7 @@
         <v>400</v>
       </c>
       <c r="E22" t="n">
-        <v>356</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23">
@@ -15634,7 +15634,7 @@
         <v>312</v>
       </c>
       <c r="E23" t="n">
-        <v>278</v>
+        <v>255</v>
       </c>
     </row>
     <row r="24">
@@ -15655,7 +15655,7 @@
         <v>163</v>
       </c>
       <c r="E24" t="n">
-        <v>145</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25">
@@ -15676,7 +15676,7 @@
         <v>1787</v>
       </c>
       <c r="E25" t="n">
-        <v>1589</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="26">
@@ -15697,7 +15697,7 @@
         <v>1348</v>
       </c>
       <c r="E26" t="n">
-        <v>1198</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="27">
@@ -15718,7 +15718,7 @@
         <v>1160</v>
       </c>
       <c r="E27" t="n">
-        <v>1032</v>
+        <v>946</v>
       </c>
     </row>
     <row r="28">
@@ -15739,7 +15739,7 @@
         <v>1624</v>
       </c>
       <c r="E28" t="n">
-        <v>1443</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="29">
@@ -15760,7 +15760,7 @@
         <v>11859</v>
       </c>
       <c r="E29" t="n">
-        <v>10543</v>
+        <v>9672</v>
       </c>
     </row>
     <row r="30">
@@ -15781,7 +15781,7 @@
         <v>1704</v>
       </c>
       <c r="E30" t="n">
-        <v>1515</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="31">
@@ -15802,7 +15802,7 @@
         <v>1610</v>
       </c>
       <c r="E31" t="n">
-        <v>1431</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="32">
@@ -15823,7 +15823,7 @@
         <v>1579</v>
       </c>
       <c r="E32" t="n">
-        <v>1403</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="33">
@@ -15844,7 +15844,7 @@
         <v>672</v>
       </c>
       <c r="E33" t="n">
-        <v>597</v>
+        <v>548</v>
       </c>
     </row>
     <row r="34">
@@ -15865,7 +15865,7 @@
         <v>668</v>
       </c>
       <c r="E34" t="n">
-        <v>594</v>
+        <v>545</v>
       </c>
     </row>
     <row r="35">
@@ -15886,7 +15886,7 @@
         <v>500</v>
       </c>
       <c r="E35" t="n">
-        <v>445</v>
+        <v>408</v>
       </c>
     </row>
     <row r="36">
@@ -15907,7 +15907,7 @@
         <v>390</v>
       </c>
       <c r="E36" t="n">
-        <v>347</v>
+        <v>318</v>
       </c>
     </row>
     <row r="37">
@@ -15928,7 +15928,7 @@
         <v>204</v>
       </c>
       <c r="E37" t="n">
-        <v>181</v>
+        <v>166</v>
       </c>
     </row>
     <row r="38">
@@ -15949,7 +15949,7 @@
         <v>2234</v>
       </c>
       <c r="E38" t="n">
-        <v>1986</v>
+        <v>1822</v>
       </c>
     </row>
     <row r="39">
@@ -15970,7 +15970,7 @@
         <v>1685</v>
       </c>
       <c r="E39" t="n">
-        <v>1498</v>
+        <v>1374</v>
       </c>
     </row>
     <row r="40">
@@ -15991,7 +15991,7 @@
         <v>1451</v>
       </c>
       <c r="E40" t="n">
-        <v>1290</v>
+        <v>1183</v>
       </c>
     </row>
     <row r="41">
@@ -16012,7 +16012,7 @@
         <v>2030</v>
       </c>
       <c r="E41" t="n">
-        <v>1804</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="42">
@@ -16033,7 +16033,7 @@
         <v>14726</v>
       </c>
       <c r="E42" t="n">
-        <v>13091</v>
+        <v>12011</v>
       </c>
     </row>
     <row r="43"/>
@@ -16074,7 +16074,7 @@
         <v>110</v>
       </c>
       <c r="E45" t="n">
-        <v>5262</v>
+        <v>4828</v>
       </c>
     </row>
     <row r="46">
@@ -16091,7 +16091,7 @@
         <v>108</v>
       </c>
       <c r="E46" t="n">
-        <v>6537</v>
+        <v>5997</v>
       </c>
     </row>
     <row r="47">
@@ -16108,7 +16108,7 @@
         <v>116</v>
       </c>
       <c r="E47" t="n">
-        <v>9282</v>
+        <v>8515</v>
       </c>
     </row>
   </sheetData>

</xml_diff>